<commit_message>
Added gif animator and assets
</commit_message>
<xml_diff>
--- a/images/image manifest.xlsx
+++ b/images/image manifest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Github\CS-Graphics\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C84FA5-8A46-47BD-BCC9-9D751975EC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D8C480-1220-47B1-B455-836D118CF091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21480" windowHeight="11520" xr2:uid="{620D0F7A-D0D3-4EA0-8A4D-C0BB25CE06A6}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="919">
   <si>
     <t>Filename</t>
   </si>
@@ -2776,6 +2776,24 @@
   </si>
   <si>
     <t>TODO(Name) Death animation</t>
+  </si>
+  <si>
+    <t>Animation stacked</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Tola healthy idle</t>
+  </si>
+  <si>
+    <t>Status bar</t>
+  </si>
+  <si>
+    <t>Tola warning idle</t>
+  </si>
+  <si>
+    <t>Tola danger idle</t>
   </si>
 </sst>
 </file>
@@ -2836,16 +2854,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D76A0E2E-5EF1-4C76-B441-AB9216212B3A}" name="Table1" displayName="Table1" ref="A1:G900" totalsRowShown="0">
-  <autoFilter ref="A1:G900" xr:uid="{D76A0E2E-5EF1-4C76-B441-AB9216212B3A}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:F869">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D76A0E2E-5EF1-4C76-B441-AB9216212B3A}" name="Table1" displayName="Table1" ref="A1:H900" totalsRowShown="0">
+  <autoFilter ref="A1:H900" xr:uid="{D76A0E2E-5EF1-4C76-B441-AB9216212B3A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:G869">
     <sortCondition ref="A1:A900"/>
   </sortState>
-  <tableColumns count="7">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5BE264B2-3040-4E26-A5F7-09EDCD3E654D}" name="Filename"/>
     <tableColumn id="2" xr3:uid="{AA34CE9E-8179-4C54-86B6-0527AB82EA40}" name="Size" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{67331664-BB23-4B18-BAE5-9C442B93DC80}" name="Palette"/>
     <tableColumn id="4" xr3:uid="{939C3ADC-1918-446F-8F03-0323F831EA15}" name="Frames"/>
+    <tableColumn id="8" xr3:uid="{9479E81C-320D-4A48-BCAE-E8694A4258D2}" name="Animation stacked"/>
     <tableColumn id="5" xr3:uid="{38C11265-21A9-4D92-ADAC-81770284CD74}" name="Type"/>
     <tableColumn id="6" xr3:uid="{E8D6B3ED-E7AB-4418-98DF-3F96091191AB}" name="Description"/>
     <tableColumn id="7" xr3:uid="{12717EBE-E94A-4C45-AE7E-ADDEC9F71820}" name="Purpose"/>
@@ -3171,17 +3190,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847C270E-F408-4D3B-B2DA-3B018BAD355D}">
-  <dimension ref="A1:G900"/>
+  <dimension ref="A1:H900"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3195,16 +3215,19 @@
         <v>5</v>
       </c>
       <c r="E1" t="s">
+        <v>913</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>910</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>752</v>
       </c>
@@ -3212,7 +3235,7 @@
         <v>75376</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>753</v>
       </c>
@@ -3220,7 +3243,7 @@
         <v>129265</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>754</v>
       </c>
@@ -3228,7 +3251,7 @@
         <v>35736</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>755</v>
       </c>
@@ -3236,7 +3259,7 @@
         <v>17697</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>756</v>
       </c>
@@ -3244,31 +3267,85 @@
         <v>50366</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1">
         <v>6370</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>909</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>914</v>
+      </c>
+      <c r="F7" t="s">
+        <v>908</v>
+      </c>
+      <c r="G7" t="s">
+        <v>915</v>
+      </c>
+      <c r="H7" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1">
         <v>20545</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>909</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>914</v>
+      </c>
+      <c r="F8" t="s">
+        <v>908</v>
+      </c>
+      <c r="G8" t="s">
+        <v>917</v>
+      </c>
+      <c r="H8" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="1">
         <v>12833</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>909</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>914</v>
+      </c>
+      <c r="F9" t="s">
+        <v>908</v>
+      </c>
+      <c r="G9" t="s">
+        <v>918</v>
+      </c>
+      <c r="H9" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3281,17 +3358,17 @@
       <c r="D10">
         <v>4</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>908</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>912</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -3299,7 +3376,7 @@
         <v>3837</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -3307,7 +3384,7 @@
         <v>17892</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -3315,7 +3392,7 @@
         <v>19255</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -3328,17 +3405,17 @@
       <c r="D14">
         <v>4</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>908</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>912</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -3346,7 +3423,7 @@
         <v>4962</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -3354,7 +3431,7 @@
         <v>27484</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -3362,7 +3439,7 @@
         <v>28958</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -3375,17 +3452,17 @@
       <c r="D18">
         <v>4</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>908</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>912</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -3393,7 +3470,7 @@
         <v>4760</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -3401,7 +3478,7 @@
         <v>18746</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -3409,7 +3486,7 @@
         <v>17387</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -3422,17 +3499,17 @@
       <c r="D22">
         <v>4</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>908</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>912</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -3440,7 +3517,7 @@
         <v>4613</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -3448,7 +3525,7 @@
         <v>18010</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -3456,7 +3533,7 @@
         <v>21511</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -3469,17 +3546,17 @@
       <c r="D26">
         <v>4</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>908</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>912</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -3487,7 +3564,7 @@
         <v>4056</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -3495,7 +3572,7 @@
         <v>26577</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -3503,7 +3580,7 @@
         <v>20293</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -3516,17 +3593,17 @@
       <c r="D30">
         <v>4</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>908</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>912</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -3534,7 +3611,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -3542,7 +3619,7 @@
         <v>18509</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -3550,7 +3627,7 @@
         <v>30532</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -3563,17 +3640,17 @@
       <c r="D34">
         <v>4</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>908</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>912</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -3581,7 +3658,7 @@
         <v>5475</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -3589,7 +3666,7 @@
         <v>23999</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -3597,7 +3674,7 @@
         <v>14302</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -3610,17 +3687,17 @@
       <c r="D38">
         <v>4</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>908</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>912</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -3628,7 +3705,7 @@
         <v>5028</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -3636,7 +3713,7 @@
         <v>14517</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -3644,7 +3721,7 @@
         <v>28308</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -3657,17 +3734,17 @@
       <c r="D42">
         <v>4</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>908</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>912</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -3675,7 +3752,7 @@
         <v>3841</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -3683,7 +3760,7 @@
         <v>13899</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -3691,7 +3768,7 @@
         <v>14453</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -3704,17 +3781,17 @@
       <c r="D46">
         <v>4</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>908</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>912</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -3722,7 +3799,7 @@
         <v>4674</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -3730,7 +3807,7 @@
         <v>8011</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -3738,7 +3815,7 @@
         <v>14578</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -3751,17 +3828,17 @@
       <c r="D50">
         <v>4</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>908</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>912</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -3769,7 +3846,7 @@
         <v>3811</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -3777,7 +3854,7 @@
         <v>16595</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -3785,7 +3862,7 @@
         <v>19139</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -3798,17 +3875,17 @@
       <c r="D54">
         <v>4</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>908</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>912</v>
       </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -3816,7 +3893,7 @@
         <v>4255</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -3824,7 +3901,7 @@
         <v>21576</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -3832,7 +3909,7 @@
         <v>20087</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -3845,17 +3922,17 @@
       <c r="D58">
         <v>4</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
         <v>908</v>
       </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
         <v>912</v>
       </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -3863,7 +3940,7 @@
         <v>3585</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -3871,7 +3948,7 @@
         <v>16072</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -3879,7 +3956,7 @@
         <v>9368</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>61</v>
       </c>
@@ -3892,17 +3969,17 @@
       <c r="D62">
         <v>4</v>
       </c>
-      <c r="E62" t="s">
+      <c r="F62" t="s">
         <v>908</v>
       </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
         <v>912</v>
       </c>
-      <c r="G62" t="s">
+      <c r="H62" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>62</v>
       </c>
@@ -3910,7 +3987,7 @@
         <v>4241</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -3918,7 +3995,7 @@
         <v>14284</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>64</v>
       </c>
@@ -3926,7 +4003,7 @@
         <v>16266</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>65</v>
       </c>
@@ -3939,17 +4016,17 @@
       <c r="D66">
         <v>4</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
         <v>908</v>
       </c>
-      <c r="F66" t="s">
+      <c r="G66" t="s">
         <v>912</v>
       </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -3957,7 +4034,7 @@
         <v>3848</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -3965,7 +4042,7 @@
         <v>14535</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -3973,7 +4050,7 @@
         <v>13543</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -3986,17 +4063,17 @@
       <c r="D70">
         <v>4</v>
       </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>908</v>
       </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>912</v>
       </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -4004,7 +4081,7 @@
         <v>4113</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -4012,7 +4089,7 @@
         <v>22095</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -4020,7 +4097,7 @@
         <v>10361</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -4033,17 +4110,17 @@
       <c r="D74">
         <v>4</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
         <v>908</v>
       </c>
-      <c r="F74" t="s">
+      <c r="G74" t="s">
         <v>912</v>
       </c>
-      <c r="G74" t="s">
+      <c r="H74" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -4051,7 +4128,7 @@
         <v>5462</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -4059,7 +4136,7 @@
         <v>16262</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -4067,7 +4144,7 @@
         <v>22865</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -4080,17 +4157,17 @@
       <c r="D78">
         <v>4</v>
       </c>
-      <c r="E78" t="s">
+      <c r="F78" t="s">
         <v>908</v>
       </c>
-      <c r="F78" t="s">
+      <c r="G78" t="s">
         <v>912</v>
       </c>
-      <c r="G78" t="s">
+      <c r="H78" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -4098,7 +4175,7 @@
         <v>3708</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -4106,7 +4183,7 @@
         <v>12093</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>80</v>
       </c>
@@ -4114,7 +4191,7 @@
         <v>22277</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>81</v>
       </c>
@@ -4127,17 +4204,17 @@
       <c r="D82">
         <v>4</v>
       </c>
-      <c r="E82" t="s">
+      <c r="F82" t="s">
         <v>908</v>
       </c>
-      <c r="F82" t="s">
+      <c r="G82" t="s">
         <v>912</v>
       </c>
-      <c r="G82" t="s">
+      <c r="H82" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>82</v>
       </c>
@@ -4145,7 +4222,7 @@
         <v>3975</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -4153,7 +4230,7 @@
         <v>20506</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -4161,7 +4238,7 @@
         <v>33413</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>85</v>
       </c>
@@ -4174,17 +4251,17 @@
       <c r="D86">
         <v>4</v>
       </c>
-      <c r="E86" t="s">
+      <c r="F86" t="s">
         <v>908</v>
       </c>
-      <c r="F86" t="s">
+      <c r="G86" t="s">
         <v>912</v>
       </c>
-      <c r="G86" t="s">
+      <c r="H86" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>86</v>
       </c>
@@ -4192,7 +4269,7 @@
         <v>6827</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>87</v>
       </c>
@@ -4200,7 +4277,7 @@
         <v>15644</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>88</v>
       </c>
@@ -4208,7 +4285,7 @@
         <v>10144</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>89</v>
       </c>
@@ -4221,17 +4298,17 @@
       <c r="D90">
         <v>4</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>908</v>
       </c>
-      <c r="F90" t="s">
+      <c r="G90" t="s">
         <v>912</v>
       </c>
-      <c r="G90" t="s">
+      <c r="H90" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -4239,7 +4316,7 @@
         <v>3942</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>91</v>
       </c>
@@ -4247,7 +4324,7 @@
         <v>25907</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>92</v>
       </c>
@@ -4255,7 +4332,7 @@
         <v>17779</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>93</v>
       </c>
@@ -4268,17 +4345,17 @@
       <c r="D94">
         <v>4</v>
       </c>
-      <c r="E94" t="s">
+      <c r="F94" t="s">
         <v>908</v>
       </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
         <v>912</v>
       </c>
-      <c r="G94" t="s">
+      <c r="H94" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>94</v>
       </c>
@@ -4286,7 +4363,7 @@
         <v>4141</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>95</v>
       </c>
@@ -4294,7 +4371,7 @@
         <v>7629</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>96</v>
       </c>
@@ -4302,7 +4379,7 @@
         <v>10819</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>97</v>
       </c>
@@ -4315,17 +4392,17 @@
       <c r="D98">
         <v>4</v>
       </c>
-      <c r="E98" t="s">
+      <c r="F98" t="s">
         <v>908</v>
       </c>
-      <c r="F98" t="s">
+      <c r="G98" t="s">
         <v>912</v>
       </c>
-      <c r="G98" t="s">
+      <c r="H98" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>98</v>
       </c>
@@ -4333,7 +4410,7 @@
         <v>3552</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>99</v>
       </c>
@@ -4341,7 +4418,7 @@
         <v>14723</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>100</v>
       </c>
@@ -4349,7 +4426,7 @@
         <v>9891</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>101</v>
       </c>
@@ -4362,17 +4439,17 @@
       <c r="D102">
         <v>4</v>
       </c>
-      <c r="E102" t="s">
+      <c r="F102" t="s">
         <v>908</v>
       </c>
-      <c r="F102" t="s">
+      <c r="G102" t="s">
         <v>912</v>
       </c>
-      <c r="G102" t="s">
+      <c r="H102" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>102</v>
       </c>
@@ -4380,7 +4457,7 @@
         <v>12582</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>103</v>
       </c>
@@ -4388,7 +4465,7 @@
         <v>15891</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>104</v>
       </c>
@@ -4396,7 +4473,7 @@
         <v>17579</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>105</v>
       </c>
@@ -4409,17 +4486,17 @@
       <c r="D106">
         <v>4</v>
       </c>
-      <c r="E106" t="s">
+      <c r="F106" t="s">
         <v>908</v>
       </c>
-      <c r="F106" t="s">
+      <c r="G106" t="s">
         <v>912</v>
       </c>
-      <c r="G106" t="s">
+      <c r="H106" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>106</v>
       </c>
@@ -4427,7 +4504,7 @@
         <v>3307</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>107</v>
       </c>
@@ -4435,7 +4512,7 @@
         <v>26686</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>108</v>
       </c>
@@ -4443,7 +4520,7 @@
         <v>14228</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>109</v>
       </c>
@@ -4456,17 +4533,17 @@
       <c r="D110">
         <v>4</v>
       </c>
-      <c r="E110" t="s">
+      <c r="F110" t="s">
         <v>908</v>
       </c>
-      <c r="F110" t="s">
+      <c r="G110" t="s">
         <v>912</v>
       </c>
-      <c r="G110" t="s">
+      <c r="H110" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>110</v>
       </c>
@@ -4474,7 +4551,7 @@
         <v>3359</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>111</v>
       </c>
@@ -4482,7 +4559,7 @@
         <v>18248</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>112</v>
       </c>
@@ -4490,7 +4567,7 @@
         <v>13247</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>113</v>
       </c>
@@ -4503,17 +4580,17 @@
       <c r="D114">
         <v>4</v>
       </c>
-      <c r="E114" t="s">
+      <c r="F114" t="s">
         <v>908</v>
       </c>
-      <c r="F114" t="s">
+      <c r="G114" t="s">
         <v>912</v>
       </c>
-      <c r="G114" t="s">
+      <c r="H114" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>114</v>
       </c>
@@ -4521,7 +4598,7 @@
         <v>3928</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>115</v>
       </c>
@@ -4529,7 +4606,7 @@
         <v>13748</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>116</v>
       </c>
@@ -4537,7 +4614,7 @@
         <v>14399</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>117</v>
       </c>
@@ -4550,17 +4627,17 @@
       <c r="D118">
         <v>4</v>
       </c>
-      <c r="E118" t="s">
+      <c r="F118" t="s">
         <v>908</v>
       </c>
-      <c r="F118" t="s">
+      <c r="G118" t="s">
         <v>912</v>
       </c>
-      <c r="G118" t="s">
+      <c r="H118" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>118</v>
       </c>
@@ -4568,7 +4645,7 @@
         <v>4177</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>119</v>
       </c>
@@ -4576,7 +4653,7 @@
         <v>17458</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>120</v>
       </c>
@@ -4584,7 +4661,7 @@
         <v>22349</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>121</v>
       </c>
@@ -4597,17 +4674,17 @@
       <c r="D122">
         <v>4</v>
       </c>
-      <c r="E122" t="s">
+      <c r="F122" t="s">
         <v>908</v>
       </c>
-      <c r="F122" t="s">
+      <c r="G122" t="s">
         <v>912</v>
       </c>
-      <c r="G122" t="s">
+      <c r="H122" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>122</v>
       </c>
@@ -4615,7 +4692,7 @@
         <v>3728</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>123</v>
       </c>
@@ -4623,7 +4700,7 @@
         <v>20617</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>124</v>
       </c>
@@ -4631,7 +4708,7 @@
         <v>14916</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>125</v>
       </c>
@@ -4644,17 +4721,17 @@
       <c r="D126">
         <v>4</v>
       </c>
-      <c r="E126" t="s">
+      <c r="F126" t="s">
         <v>908</v>
       </c>
-      <c r="F126" t="s">
+      <c r="G126" t="s">
         <v>912</v>
       </c>
-      <c r="G126" t="s">
+      <c r="H126" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>126</v>
       </c>
@@ -4662,7 +4739,7 @@
         <v>5462</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>127</v>
       </c>
@@ -4670,7 +4747,7 @@
         <v>16262</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>128</v>
       </c>
@@ -4678,7 +4755,7 @@
         <v>22865</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>129</v>
       </c>
@@ -4691,17 +4768,17 @@
       <c r="D130">
         <v>4</v>
       </c>
-      <c r="E130" t="s">
+      <c r="F130" t="s">
         <v>908</v>
       </c>
-      <c r="F130" t="s">
+      <c r="G130" t="s">
         <v>912</v>
       </c>
-      <c r="G130" t="s">
+      <c r="H130" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>757</v>
       </c>
@@ -4709,7 +4786,7 @@
         <v>19481</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>758</v>
       </c>
@@ -4717,7 +4794,7 @@
         <v>25838</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>759</v>
       </c>
@@ -4725,7 +4802,7 @@
         <v>15438</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>760</v>
       </c>
@@ -4733,7 +4810,7 @@
         <v>1434824</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>761</v>
       </c>
@@ -4741,7 +4818,7 @@
         <v>2086653</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>762</v>
       </c>
@@ -4749,7 +4826,7 @@
         <v>1007413</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>763</v>
       </c>
@@ -4757,7 +4834,7 @@
         <v>50601</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>764</v>
       </c>
@@ -4765,7 +4842,7 @@
         <v>164306</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>765</v>
       </c>
@@ -4773,7 +4850,7 @@
         <v>663860</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>766</v>
       </c>
@@ -4781,7 +4858,7 @@
         <v>739003</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>767</v>
       </c>
@@ -4789,7 +4866,7 @@
         <v>665272</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>768</v>
       </c>
@@ -4797,7 +4874,7 @@
         <v>635163</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>769</v>
       </c>
@@ -4805,7 +4882,7 @@
         <v>760300</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>770</v>
       </c>
@@ -10829,7 +10906,7 @@
         <v>757884</v>
       </c>
     </row>
-    <row r="897" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="897" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A897" t="s">
         <v>904</v>
       </c>
@@ -10842,14 +10919,14 @@
       <c r="D897">
         <v>1</v>
       </c>
-      <c r="E897" t="s">
+      <c r="F897" t="s">
         <v>906</v>
       </c>
-      <c r="F897" t="s">
+      <c r="G897" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="898" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="898" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A898" t="s">
         <v>901</v>
       </c>
@@ -10857,7 +10934,7 @@
         <v>2851</v>
       </c>
     </row>
-    <row r="899" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="899" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A899" t="s">
         <v>902</v>
       </c>
@@ -10865,7 +10942,7 @@
         <v>186389</v>
       </c>
     </row>
-    <row r="900" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="900" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A900" t="s">
         <v>903</v>
       </c>

</xml_diff>

<commit_message>
Added more sprites, Shadow
</commit_message>
<xml_diff>
--- a/images/image manifest.xlsx
+++ b/images/image manifest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Github\CS-Graphics\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2911D216-6E45-4439-87FA-BD143F5C5F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B09CAA-8A69-4A9F-B34C-666860D8A036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="810" windowWidth="21600" windowHeight="11295" xr2:uid="{620D0F7A-D0D3-4EA0-8A4D-C0BB25CE06A6}"/>
+    <workbookView xWindow="4905" yWindow="2730" windowWidth="15930" windowHeight="8145" xr2:uid="{620D0F7A-D0D3-4EA0-8A4D-C0BB25CE06A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2290" uniqueCount="981">
   <si>
     <t>Filename</t>
   </si>
@@ -2824,6 +2824,162 @@
   </si>
   <si>
     <t>TODO(Name) danger idle</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Red Hex background</t>
+  </si>
+  <si>
+    <t>Layer behind game hex tiles</t>
+  </si>
+  <si>
+    <t>Green Hex background</t>
+  </si>
+  <si>
+    <t>Battle FX</t>
+  </si>
+  <si>
+    <t>Mushroom cloud explosion</t>
+  </si>
+  <si>
+    <t>Explosion</t>
+  </si>
+  <si>
+    <t>Nova Explosion</t>
+  </si>
+  <si>
+    <t>Orb</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Shields</t>
+  </si>
+  <si>
+    <t>Blue Plasma Ball</t>
+  </si>
+  <si>
+    <t>Red Plasma Ball</t>
+  </si>
+  <si>
+    <t>Flair</t>
+  </si>
+  <si>
+    <t>Directional Projectile</t>
+  </si>
+  <si>
+    <t>Long Directional Projectile</t>
+  </si>
+  <si>
+    <t>Wide Directional Projectile</t>
+  </si>
+  <si>
+    <t>Short Directional Projectile</t>
+  </si>
+  <si>
+    <t>Missile Projectile</t>
+  </si>
+  <si>
+    <t>Smoke</t>
+  </si>
+  <si>
+    <t>Sphere</t>
+  </si>
+  <si>
+    <t>SIMGUI.PLX</t>
+  </si>
+  <si>
+    <t>Crouched man with sword</t>
+  </si>
+  <si>
+    <t>TODO (Label)</t>
+  </si>
+  <si>
+    <t>Shadow</t>
+  </si>
+  <si>
+    <t>Standing</t>
+  </si>
+  <si>
+    <t>Cadaver</t>
+  </si>
+  <si>
+    <t>Crouched</t>
+  </si>
+  <si>
+    <t>North stand to crouching</t>
+  </si>
+  <si>
+    <t>Northwest stand to crouching</t>
+  </si>
+  <si>
+    <t>Southwest stand to crouching</t>
+  </si>
+  <si>
+    <t>South stand to crouching</t>
+  </si>
+  <si>
+    <t>Southeast stand to crouching</t>
+  </si>
+  <si>
+    <t>Northeast stand to crouching</t>
+  </si>
+  <si>
+    <t>Northwest jump</t>
+  </si>
+  <si>
+    <t>North jump</t>
+  </si>
+  <si>
+    <t>Southwest jump</t>
+  </si>
+  <si>
+    <t>South jump</t>
+  </si>
+  <si>
+    <t>Southeast jump</t>
+  </si>
+  <si>
+    <t>Northeast jump</t>
+  </si>
+  <si>
+    <t>North walk short</t>
+  </si>
+  <si>
+    <t>Northwest walk short</t>
+  </si>
+  <si>
+    <t>Southwest walk short</t>
+  </si>
+  <si>
+    <t>South walk short</t>
+  </si>
+  <si>
+    <t>Southeast walk short</t>
+  </si>
+  <si>
+    <t>Northeast walk short</t>
+  </si>
+  <si>
+    <t>Northwest walk long</t>
+  </si>
+  <si>
+    <t>Southwest walk long</t>
+  </si>
+  <si>
+    <t>South walk long</t>
+  </si>
+  <si>
+    <t>Southeast walk long</t>
+  </si>
+  <si>
+    <t>Northeast walk long</t>
+  </si>
+  <si>
+    <t>North walk long</t>
   </si>
 </sst>
 </file>
@@ -3226,6 +3382,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="9.85546875" customWidth="1"/>
@@ -3320,6 +3477,30 @@
       <c r="B5" s="1">
         <v>17697</v>
       </c>
+      <c r="C5" t="s">
+        <v>909</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>919</v>
+      </c>
+      <c r="F5" t="s">
+        <v>919</v>
+      </c>
+      <c r="G5" t="s">
+        <v>919</v>
+      </c>
+      <c r="H5" t="s">
+        <v>929</v>
+      </c>
+      <c r="I5" t="s">
+        <v>932</v>
+      </c>
+      <c r="J5" t="s">
+        <v>931</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -7203,6 +7384,9 @@
       <c r="F130" t="s">
         <v>919</v>
       </c>
+      <c r="G130" t="s">
+        <v>919</v>
+      </c>
       <c r="H130" t="s">
         <v>908</v>
       </c>
@@ -7220,6 +7404,30 @@
       <c r="B131" s="1">
         <v>19481</v>
       </c>
+      <c r="C131" t="s">
+        <v>909</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131" t="s">
+        <v>919</v>
+      </c>
+      <c r="F131" t="s">
+        <v>919</v>
+      </c>
+      <c r="G131" t="s">
+        <v>919</v>
+      </c>
+      <c r="H131" t="s">
+        <v>929</v>
+      </c>
+      <c r="I131" t="s">
+        <v>930</v>
+      </c>
+      <c r="J131" t="s">
+        <v>931</v>
+      </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
@@ -7581,7 +7789,7 @@
         <v>4102</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>803</v>
       </c>
@@ -7589,7 +7797,7 @@
         <v>1749</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>804</v>
       </c>
@@ -7597,7 +7805,7 @@
         <v>10895</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>805</v>
       </c>
@@ -7605,191 +7813,671 @@
         <v>16865</v>
       </c>
     </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>806</v>
       </c>
       <c r="B180" s="1">
         <v>9019</v>
       </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C180" t="s">
+        <v>909</v>
+      </c>
+      <c r="D180">
+        <v>15</v>
+      </c>
+      <c r="E180" t="s">
+        <v>914</v>
+      </c>
+      <c r="F180" t="s">
+        <v>919</v>
+      </c>
+      <c r="G180" t="s">
+        <v>919</v>
+      </c>
+      <c r="H180" t="s">
+        <v>933</v>
+      </c>
+      <c r="I180" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>807</v>
       </c>
       <c r="B181" s="1">
         <v>8786</v>
       </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C181" t="s">
+        <v>909</v>
+      </c>
+      <c r="D181">
+        <v>16</v>
+      </c>
+      <c r="E181" t="s">
+        <v>914</v>
+      </c>
+      <c r="F181" t="s">
+        <v>919</v>
+      </c>
+      <c r="G181" t="s">
+        <v>919</v>
+      </c>
+      <c r="H181" t="s">
+        <v>933</v>
+      </c>
+      <c r="I181" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>808</v>
       </c>
       <c r="B182" s="1">
         <v>30883</v>
       </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C182" t="s">
+        <v>909</v>
+      </c>
+      <c r="D182">
+        <v>31</v>
+      </c>
+      <c r="E182" t="s">
+        <v>914</v>
+      </c>
+      <c r="F182" t="s">
+        <v>919</v>
+      </c>
+      <c r="G182" t="s">
+        <v>919</v>
+      </c>
+      <c r="H182" t="s">
+        <v>933</v>
+      </c>
+      <c r="I182" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>809</v>
       </c>
       <c r="B183" s="1">
         <v>16796</v>
       </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C183" t="s">
+        <v>909</v>
+      </c>
+      <c r="D183">
+        <v>15</v>
+      </c>
+      <c r="E183" t="s">
+        <v>914</v>
+      </c>
+      <c r="F183" t="s">
+        <v>919</v>
+      </c>
+      <c r="G183" t="s">
+        <v>919</v>
+      </c>
+      <c r="H183" t="s">
+        <v>933</v>
+      </c>
+      <c r="I183" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>810</v>
       </c>
       <c r="B184" s="1">
         <v>10120</v>
       </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C184" t="s">
+        <v>909</v>
+      </c>
+      <c r="D184">
+        <v>30</v>
+      </c>
+      <c r="E184" t="s">
+        <v>914</v>
+      </c>
+      <c r="F184" t="s">
+        <v>919</v>
+      </c>
+      <c r="G184" t="s">
+        <v>919</v>
+      </c>
+      <c r="H184" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>811</v>
       </c>
       <c r="B185" s="1">
         <v>15870</v>
       </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C185" t="s">
+        <v>909</v>
+      </c>
+      <c r="D185">
+        <v>15</v>
+      </c>
+      <c r="E185" t="s">
+        <v>914</v>
+      </c>
+      <c r="F185" t="s">
+        <v>919</v>
+      </c>
+      <c r="G185" t="s">
+        <v>919</v>
+      </c>
+      <c r="H185" t="s">
+        <v>933</v>
+      </c>
+      <c r="I185" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>812</v>
       </c>
       <c r="B186" s="1">
         <v>26036</v>
       </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C186" t="s">
+        <v>909</v>
+      </c>
+      <c r="D186">
+        <v>24</v>
+      </c>
+      <c r="E186" t="s">
+        <v>914</v>
+      </c>
+      <c r="F186" t="s">
+        <v>919</v>
+      </c>
+      <c r="G186" t="s">
+        <v>919</v>
+      </c>
+      <c r="H186" t="s">
+        <v>933</v>
+      </c>
+      <c r="I186" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>813</v>
       </c>
       <c r="B187" s="1">
         <v>50678</v>
       </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C187" t="s">
+        <v>909</v>
+      </c>
+      <c r="D187">
+        <v>20</v>
+      </c>
+      <c r="E187" t="s">
+        <v>914</v>
+      </c>
+      <c r="F187" t="s">
+        <v>919</v>
+      </c>
+      <c r="G187" t="s">
+        <v>919</v>
+      </c>
+      <c r="H187" t="s">
+        <v>933</v>
+      </c>
+      <c r="I187" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>814</v>
       </c>
       <c r="B188" s="1">
         <v>11718</v>
       </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C188" t="s">
+        <v>909</v>
+      </c>
+      <c r="D188">
+        <v>30</v>
+      </c>
+      <c r="E188" t="s">
+        <v>914</v>
+      </c>
+      <c r="F188" t="s">
+        <v>919</v>
+      </c>
+      <c r="G188" t="s">
+        <v>919</v>
+      </c>
+      <c r="H188" t="s">
+        <v>933</v>
+      </c>
+      <c r="I188" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>815</v>
       </c>
       <c r="B189" s="1">
         <v>8697</v>
       </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C189" t="s">
+        <v>909</v>
+      </c>
+      <c r="D189">
+        <v>11</v>
+      </c>
+      <c r="E189" t="s">
+        <v>914</v>
+      </c>
+      <c r="F189" t="s">
+        <v>919</v>
+      </c>
+      <c r="G189" t="s">
+        <v>919</v>
+      </c>
+      <c r="H189" t="s">
+        <v>933</v>
+      </c>
+      <c r="I189" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>816</v>
       </c>
       <c r="B190" s="1">
         <v>11351</v>
       </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C190" t="s">
+        <v>909</v>
+      </c>
+      <c r="D190">
+        <v>31</v>
+      </c>
+      <c r="E190" t="s">
+        <v>914</v>
+      </c>
+      <c r="F190" t="s">
+        <v>919</v>
+      </c>
+      <c r="G190" t="s">
+        <v>919</v>
+      </c>
+      <c r="H190" t="s">
+        <v>933</v>
+      </c>
+      <c r="I190" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>817</v>
       </c>
       <c r="B191" s="1">
         <v>18961</v>
       </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C191" t="s">
+        <v>909</v>
+      </c>
+      <c r="D191">
+        <v>44</v>
+      </c>
+      <c r="E191" t="s">
+        <v>914</v>
+      </c>
+      <c r="F191" t="s">
+        <v>919</v>
+      </c>
+      <c r="G191" t="s">
+        <v>919</v>
+      </c>
+      <c r="H191" t="s">
+        <v>933</v>
+      </c>
+      <c r="I191" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>818</v>
       </c>
       <c r="B192" s="1">
         <v>41109</v>
       </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C192" t="s">
+        <v>909</v>
+      </c>
+      <c r="D192">
+        <v>24</v>
+      </c>
+      <c r="E192" t="s">
+        <v>914</v>
+      </c>
+      <c r="F192" t="s">
+        <v>919</v>
+      </c>
+      <c r="G192" t="s">
+        <v>919</v>
+      </c>
+      <c r="H192" t="s">
+        <v>933</v>
+      </c>
+      <c r="I192" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>819</v>
       </c>
       <c r="B193" s="1">
         <v>1813</v>
       </c>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C193" t="s">
+        <v>909</v>
+      </c>
+      <c r="D193">
+        <v>6</v>
+      </c>
+      <c r="E193" t="s">
+        <v>914</v>
+      </c>
+      <c r="F193" t="s">
+        <v>919</v>
+      </c>
+      <c r="G193" t="s">
+        <v>919</v>
+      </c>
+      <c r="H193" t="s">
+        <v>933</v>
+      </c>
+      <c r="I193" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>820</v>
       </c>
       <c r="B194" s="1">
         <v>30736</v>
       </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C194" t="s">
+        <v>909</v>
+      </c>
+      <c r="D194">
+        <v>26</v>
+      </c>
+      <c r="E194" t="s">
+        <v>914</v>
+      </c>
+      <c r="F194" t="s">
+        <v>919</v>
+      </c>
+      <c r="G194" t="s">
+        <v>919</v>
+      </c>
+      <c r="H194" t="s">
+        <v>933</v>
+      </c>
+      <c r="I194" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>821</v>
       </c>
       <c r="B195" s="1">
         <v>89108</v>
       </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C195" t="s">
+        <v>909</v>
+      </c>
+      <c r="D195">
+        <v>31</v>
+      </c>
+      <c r="E195" t="s">
+        <v>914</v>
+      </c>
+      <c r="F195" t="s">
+        <v>919</v>
+      </c>
+      <c r="G195" t="s">
+        <v>919</v>
+      </c>
+      <c r="H195" t="s">
+        <v>933</v>
+      </c>
+      <c r="I195" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>822</v>
       </c>
       <c r="B196" s="1">
         <v>136329</v>
       </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C196" t="s">
+        <v>909</v>
+      </c>
+      <c r="D196">
+        <v>31</v>
+      </c>
+      <c r="E196" t="s">
+        <v>914</v>
+      </c>
+      <c r="F196" t="s">
+        <v>919</v>
+      </c>
+      <c r="G196" t="s">
+        <v>919</v>
+      </c>
+      <c r="H196" t="s">
+        <v>933</v>
+      </c>
+      <c r="I196" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>823</v>
       </c>
       <c r="B197" s="1">
         <v>40852</v>
       </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C197" t="s">
+        <v>909</v>
+      </c>
+      <c r="D197">
+        <v>31</v>
+      </c>
+      <c r="E197" t="s">
+        <v>914</v>
+      </c>
+      <c r="F197" t="s">
+        <v>919</v>
+      </c>
+      <c r="G197" t="s">
+        <v>919</v>
+      </c>
+      <c r="H197" t="s">
+        <v>933</v>
+      </c>
+      <c r="I197" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>824</v>
       </c>
       <c r="B198" s="1">
         <v>84638</v>
       </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C198" t="s">
+        <v>909</v>
+      </c>
+      <c r="D198">
+        <v>31</v>
+      </c>
+      <c r="E198" t="s">
+        <v>914</v>
+      </c>
+      <c r="F198" t="s">
+        <v>919</v>
+      </c>
+      <c r="G198" t="s">
+        <v>919</v>
+      </c>
+      <c r="H198" t="s">
+        <v>933</v>
+      </c>
+      <c r="I198" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>825</v>
       </c>
       <c r="B199" s="1">
         <v>21077</v>
       </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C199" t="s">
+        <v>909</v>
+      </c>
+      <c r="D199">
+        <v>29</v>
+      </c>
+      <c r="E199" t="s">
+        <v>914</v>
+      </c>
+      <c r="F199" t="s">
+        <v>919</v>
+      </c>
+      <c r="G199" t="s">
+        <v>919</v>
+      </c>
+      <c r="H199" t="s">
+        <v>933</v>
+      </c>
+      <c r="I199" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>826</v>
       </c>
       <c r="B200" s="1">
         <v>3737</v>
       </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C200" t="s">
+        <v>909</v>
+      </c>
+      <c r="D200">
+        <v>14</v>
+      </c>
+      <c r="E200" t="s">
+        <v>914</v>
+      </c>
+      <c r="F200" t="s">
+        <v>919</v>
+      </c>
+      <c r="G200" t="s">
+        <v>919</v>
+      </c>
+      <c r="H200" t="s">
+        <v>933</v>
+      </c>
+      <c r="I200" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>827</v>
       </c>
       <c r="B201" s="1">
         <v>52188</v>
       </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C201" t="s">
+        <v>909</v>
+      </c>
+      <c r="D201">
+        <v>77</v>
+      </c>
+      <c r="E201" t="s">
+        <v>914</v>
+      </c>
+      <c r="F201" t="s">
+        <v>919</v>
+      </c>
+      <c r="G201" t="s">
+        <v>919</v>
+      </c>
+      <c r="H201" t="s">
+        <v>933</v>
+      </c>
+      <c r="I201" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>828</v>
       </c>
       <c r="B202" s="1">
         <v>16624</v>
       </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C202" t="s">
+        <v>909</v>
+      </c>
+      <c r="D202">
+        <v>19</v>
+      </c>
+      <c r="E202" t="s">
+        <v>914</v>
+      </c>
+      <c r="F202" t="s">
+        <v>919</v>
+      </c>
+      <c r="G202" t="s">
+        <v>919</v>
+      </c>
+      <c r="H202" t="s">
+        <v>933</v>
+      </c>
+      <c r="I202" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>829</v>
       </c>
@@ -7797,7 +8485,7 @@
         <v>11616</v>
       </c>
     </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>830</v>
       </c>
@@ -7805,7 +8493,7 @@
         <v>21117</v>
       </c>
     </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>831</v>
       </c>
@@ -7813,303 +8501,1047 @@
         <v>14596</v>
       </c>
     </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>832</v>
       </c>
       <c r="B206" s="1">
         <v>12306</v>
       </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C206" t="s">
+        <v>909</v>
+      </c>
+      <c r="D206">
+        <v>30</v>
+      </c>
+      <c r="E206" t="s">
+        <v>914</v>
+      </c>
+      <c r="F206" t="s">
+        <v>919</v>
+      </c>
+      <c r="G206" t="s">
+        <v>919</v>
+      </c>
+      <c r="H206" t="s">
+        <v>933</v>
+      </c>
+      <c r="I206" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>833</v>
       </c>
       <c r="B207" s="1">
         <v>14881</v>
       </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C207" t="s">
+        <v>909</v>
+      </c>
+      <c r="D207">
+        <v>30</v>
+      </c>
+      <c r="E207" t="s">
+        <v>914</v>
+      </c>
+      <c r="F207" t="s">
+        <v>919</v>
+      </c>
+      <c r="G207" t="s">
+        <v>919</v>
+      </c>
+      <c r="H207" t="s">
+        <v>933</v>
+      </c>
+      <c r="I207" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>834</v>
       </c>
       <c r="B208" s="1">
         <v>15823</v>
       </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C208" t="s">
+        <v>909</v>
+      </c>
+      <c r="D208">
+        <v>30</v>
+      </c>
+      <c r="E208" t="s">
+        <v>914</v>
+      </c>
+      <c r="F208" t="s">
+        <v>919</v>
+      </c>
+      <c r="G208" t="s">
+        <v>919</v>
+      </c>
+      <c r="H208" t="s">
+        <v>933</v>
+      </c>
+      <c r="I208" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>835</v>
       </c>
       <c r="B209" s="1">
         <v>8784</v>
       </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C209" t="s">
+        <v>909</v>
+      </c>
+      <c r="D209">
+        <v>30</v>
+      </c>
+      <c r="E209" t="s">
+        <v>914</v>
+      </c>
+      <c r="F209" t="s">
+        <v>919</v>
+      </c>
+      <c r="G209" t="s">
+        <v>919</v>
+      </c>
+      <c r="H209" t="s">
+        <v>933</v>
+      </c>
+      <c r="I209" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>836</v>
       </c>
       <c r="B210">
         <v>758</v>
       </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C210" t="s">
+        <v>909</v>
+      </c>
+      <c r="D210">
+        <v>12</v>
+      </c>
+      <c r="E210" t="s">
+        <v>914</v>
+      </c>
+      <c r="F210" t="s">
+        <v>919</v>
+      </c>
+      <c r="G210" t="s">
+        <v>919</v>
+      </c>
+      <c r="H210" t="s">
+        <v>933</v>
+      </c>
+      <c r="I210" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>837</v>
       </c>
       <c r="B211">
         <v>642</v>
       </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C211" t="s">
+        <v>909</v>
+      </c>
+      <c r="D211">
+        <v>12</v>
+      </c>
+      <c r="E211" t="s">
+        <v>914</v>
+      </c>
+      <c r="F211" t="s">
+        <v>919</v>
+      </c>
+      <c r="G211" t="s">
+        <v>919</v>
+      </c>
+      <c r="H211" t="s">
+        <v>933</v>
+      </c>
+      <c r="I211" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>838</v>
       </c>
       <c r="B212" s="1">
         <v>7574</v>
       </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C212" t="s">
+        <v>909</v>
+      </c>
+      <c r="D212">
+        <v>24</v>
+      </c>
+      <c r="E212" t="s">
+        <v>914</v>
+      </c>
+      <c r="F212" t="s">
+        <v>919</v>
+      </c>
+      <c r="G212" t="s">
+        <v>919</v>
+      </c>
+      <c r="H212" t="s">
+        <v>933</v>
+      </c>
+      <c r="I212" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>839</v>
       </c>
       <c r="B213" s="1">
         <v>3884</v>
       </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C213" t="s">
+        <v>909</v>
+      </c>
+      <c r="D213">
+        <v>25</v>
+      </c>
+      <c r="E213" t="s">
+        <v>914</v>
+      </c>
+      <c r="F213" t="s">
+        <v>919</v>
+      </c>
+      <c r="G213" t="s">
+        <v>919</v>
+      </c>
+      <c r="H213" t="s">
+        <v>933</v>
+      </c>
+      <c r="I213" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>840</v>
       </c>
       <c r="B214" s="1">
         <v>2475</v>
       </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C214" t="s">
+        <v>909</v>
+      </c>
+      <c r="D214">
+        <v>25</v>
+      </c>
+      <c r="E214" t="s">
+        <v>914</v>
+      </c>
+      <c r="F214" t="s">
+        <v>919</v>
+      </c>
+      <c r="G214" t="s">
+        <v>919</v>
+      </c>
+      <c r="H214" t="s">
+        <v>933</v>
+      </c>
+      <c r="I214" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>841</v>
       </c>
       <c r="B215" s="1">
         <v>1318</v>
       </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C215" t="s">
+        <v>909</v>
+      </c>
+      <c r="D215">
+        <v>24</v>
+      </c>
+      <c r="E215" t="s">
+        <v>919</v>
+      </c>
+      <c r="F215" t="s">
+        <v>919</v>
+      </c>
+      <c r="G215" t="s">
+        <v>914</v>
+      </c>
+      <c r="H215" t="s">
+        <v>933</v>
+      </c>
+      <c r="I215" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>842</v>
       </c>
       <c r="B216" s="1">
         <v>1178</v>
       </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C216" t="s">
+        <v>909</v>
+      </c>
+      <c r="D216">
+        <v>24</v>
+      </c>
+      <c r="E216" t="s">
+        <v>919</v>
+      </c>
+      <c r="F216" t="s">
+        <v>919</v>
+      </c>
+      <c r="G216" t="s">
+        <v>914</v>
+      </c>
+      <c r="H216" t="s">
+        <v>933</v>
+      </c>
+      <c r="I216" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>843</v>
       </c>
       <c r="B217" s="1">
         <v>1263</v>
       </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C217" t="s">
+        <v>909</v>
+      </c>
+      <c r="D217">
+        <v>24</v>
+      </c>
+      <c r="E217" t="s">
+        <v>919</v>
+      </c>
+      <c r="F217" t="s">
+        <v>919</v>
+      </c>
+      <c r="G217" t="s">
+        <v>914</v>
+      </c>
+      <c r="H217" t="s">
+        <v>933</v>
+      </c>
+      <c r="I217" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>844</v>
       </c>
       <c r="B218" s="1">
         <v>1210</v>
       </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C218" t="s">
+        <v>909</v>
+      </c>
+      <c r="D218">
+        <v>24</v>
+      </c>
+      <c r="E218" t="s">
+        <v>919</v>
+      </c>
+      <c r="F218" t="s">
+        <v>919</v>
+      </c>
+      <c r="G218" t="s">
+        <v>914</v>
+      </c>
+      <c r="H218" t="s">
+        <v>933</v>
+      </c>
+      <c r="I218" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>845</v>
       </c>
       <c r="B219" s="1">
         <v>9002</v>
       </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C219" t="s">
+        <v>909</v>
+      </c>
+      <c r="D219">
+        <v>24</v>
+      </c>
+      <c r="E219" t="s">
+        <v>919</v>
+      </c>
+      <c r="F219" t="s">
+        <v>919</v>
+      </c>
+      <c r="G219" t="s">
+        <v>914</v>
+      </c>
+      <c r="H219" t="s">
+        <v>933</v>
+      </c>
+      <c r="I219" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>846</v>
       </c>
       <c r="B220" s="1">
         <v>1233</v>
       </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C220" t="s">
+        <v>909</v>
+      </c>
+      <c r="D220">
+        <v>24</v>
+      </c>
+      <c r="E220" t="s">
+        <v>919</v>
+      </c>
+      <c r="F220" t="s">
+        <v>919</v>
+      </c>
+      <c r="G220" t="s">
+        <v>914</v>
+      </c>
+      <c r="H220" t="s">
+        <v>933</v>
+      </c>
+      <c r="I220" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>847</v>
       </c>
       <c r="B221" s="1">
         <v>1524</v>
       </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C221" t="s">
+        <v>909</v>
+      </c>
+      <c r="D221">
+        <v>24</v>
+      </c>
+      <c r="E221" t="s">
+        <v>919</v>
+      </c>
+      <c r="F221" t="s">
+        <v>919</v>
+      </c>
+      <c r="G221" t="s">
+        <v>914</v>
+      </c>
+      <c r="H221" t="s">
+        <v>933</v>
+      </c>
+      <c r="I221" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>848</v>
       </c>
       <c r="B222">
         <v>444</v>
       </c>
-    </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C222" t="s">
+        <v>909</v>
+      </c>
+      <c r="D222">
+        <v>24</v>
+      </c>
+      <c r="E222" t="s">
+        <v>919</v>
+      </c>
+      <c r="F222" t="s">
+        <v>919</v>
+      </c>
+      <c r="G222" t="s">
+        <v>914</v>
+      </c>
+      <c r="H222" t="s">
+        <v>933</v>
+      </c>
+      <c r="I222" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>849</v>
       </c>
       <c r="B223">
         <v>803</v>
       </c>
-    </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C223" t="s">
+        <v>909</v>
+      </c>
+      <c r="D223">
+        <v>24</v>
+      </c>
+      <c r="E223" t="s">
+        <v>919</v>
+      </c>
+      <c r="F223" t="s">
+        <v>919</v>
+      </c>
+      <c r="G223" t="s">
+        <v>914</v>
+      </c>
+      <c r="H223" t="s">
+        <v>933</v>
+      </c>
+      <c r="I223" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>850</v>
       </c>
       <c r="B224" s="1">
         <v>1218</v>
       </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C224" t="s">
+        <v>909</v>
+      </c>
+      <c r="D224">
+        <v>24</v>
+      </c>
+      <c r="E224" t="s">
+        <v>919</v>
+      </c>
+      <c r="F224" t="s">
+        <v>919</v>
+      </c>
+      <c r="G224" t="s">
+        <v>914</v>
+      </c>
+      <c r="H224" t="s">
+        <v>933</v>
+      </c>
+      <c r="I224" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>851</v>
       </c>
       <c r="B225">
         <v>871</v>
       </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C225" t="s">
+        <v>909</v>
+      </c>
+      <c r="D225">
+        <v>24</v>
+      </c>
+      <c r="E225" t="s">
+        <v>919</v>
+      </c>
+      <c r="F225" t="s">
+        <v>919</v>
+      </c>
+      <c r="G225" t="s">
+        <v>914</v>
+      </c>
+      <c r="H225" t="s">
+        <v>933</v>
+      </c>
+      <c r="I225" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>852</v>
       </c>
       <c r="B226">
         <v>559</v>
       </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C226" t="s">
+        <v>909</v>
+      </c>
+      <c r="D226">
+        <v>12</v>
+      </c>
+      <c r="E226" t="s">
+        <v>919</v>
+      </c>
+      <c r="F226" t="s">
+        <v>919</v>
+      </c>
+      <c r="G226" t="s">
+        <v>914</v>
+      </c>
+      <c r="H226" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>853</v>
       </c>
       <c r="B227">
         <v>618</v>
       </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C227" t="s">
+        <v>909</v>
+      </c>
+      <c r="D227">
+        <v>12</v>
+      </c>
+      <c r="E227" t="s">
+        <v>919</v>
+      </c>
+      <c r="F227" t="s">
+        <v>919</v>
+      </c>
+      <c r="G227" t="s">
+        <v>914</v>
+      </c>
+      <c r="H227" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>854</v>
       </c>
       <c r="B228">
         <v>582</v>
       </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C228" t="s">
+        <v>909</v>
+      </c>
+      <c r="D228">
+        <v>12</v>
+      </c>
+      <c r="E228" t="s">
+        <v>919</v>
+      </c>
+      <c r="F228" t="s">
+        <v>919</v>
+      </c>
+      <c r="G228" t="s">
+        <v>914</v>
+      </c>
+      <c r="H228" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>855</v>
       </c>
       <c r="B229">
         <v>411</v>
       </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C229" t="s">
+        <v>909</v>
+      </c>
+      <c r="D229">
+        <v>12</v>
+      </c>
+      <c r="E229" t="s">
+        <v>919</v>
+      </c>
+      <c r="F229" t="s">
+        <v>919</v>
+      </c>
+      <c r="G229" t="s">
+        <v>914</v>
+      </c>
+      <c r="H229" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>856</v>
       </c>
       <c r="B230">
         <v>327</v>
       </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C230" t="s">
+        <v>909</v>
+      </c>
+      <c r="D230">
+        <v>4</v>
+      </c>
+      <c r="E230" t="s">
+        <v>919</v>
+      </c>
+      <c r="F230" t="s">
+        <v>919</v>
+      </c>
+      <c r="G230" t="s">
+        <v>914</v>
+      </c>
+      <c r="H230" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>857</v>
       </c>
       <c r="B231">
         <v>310</v>
       </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C231" t="s">
+        <v>909</v>
+      </c>
+      <c r="D231">
+        <v>4</v>
+      </c>
+      <c r="E231" t="s">
+        <v>919</v>
+      </c>
+      <c r="F231" t="s">
+        <v>919</v>
+      </c>
+      <c r="G231" t="s">
+        <v>914</v>
+      </c>
+      <c r="H231" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>858</v>
       </c>
       <c r="B232">
         <v>317</v>
       </c>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C232" t="s">
+        <v>909</v>
+      </c>
+      <c r="D232">
+        <v>4</v>
+      </c>
+      <c r="E232" t="s">
+        <v>919</v>
+      </c>
+      <c r="F232" t="s">
+        <v>919</v>
+      </c>
+      <c r="G232" t="s">
+        <v>914</v>
+      </c>
+      <c r="H232" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>859</v>
       </c>
       <c r="B233">
         <v>323</v>
       </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C233" t="s">
+        <v>909</v>
+      </c>
+      <c r="D233">
+        <v>4</v>
+      </c>
+      <c r="E233" t="s">
+        <v>919</v>
+      </c>
+      <c r="F233" t="s">
+        <v>919</v>
+      </c>
+      <c r="G233" t="s">
+        <v>914</v>
+      </c>
+      <c r="H233" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>860</v>
       </c>
       <c r="B234">
         <v>316</v>
       </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C234" t="s">
+        <v>909</v>
+      </c>
+      <c r="D234">
+        <v>4</v>
+      </c>
+      <c r="E234" t="s">
+        <v>919</v>
+      </c>
+      <c r="F234" t="s">
+        <v>919</v>
+      </c>
+      <c r="G234" t="s">
+        <v>914</v>
+      </c>
+      <c r="H234" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>861</v>
       </c>
       <c r="B235">
         <v>309</v>
       </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C235" t="s">
+        <v>909</v>
+      </c>
+      <c r="D235">
+        <v>4</v>
+      </c>
+      <c r="E235" t="s">
+        <v>919</v>
+      </c>
+      <c r="F235" t="s">
+        <v>919</v>
+      </c>
+      <c r="G235" t="s">
+        <v>914</v>
+      </c>
+      <c r="H235" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>862</v>
       </c>
       <c r="B236" s="1">
         <v>3833</v>
       </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C236" t="s">
+        <v>909</v>
+      </c>
+      <c r="D236">
+        <v>93</v>
+      </c>
+      <c r="E236" t="s">
+        <v>914</v>
+      </c>
+      <c r="F236" t="s">
+        <v>919</v>
+      </c>
+      <c r="G236" t="s">
+        <v>919</v>
+      </c>
+      <c r="H236" t="s">
+        <v>933</v>
+      </c>
+      <c r="I236" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>863</v>
       </c>
       <c r="B237" s="1">
         <v>2227</v>
       </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C237" t="s">
+        <v>909</v>
+      </c>
+      <c r="D237">
+        <v>47</v>
+      </c>
+      <c r="E237" t="s">
+        <v>914</v>
+      </c>
+      <c r="F237" t="s">
+        <v>919</v>
+      </c>
+      <c r="G237" t="s">
+        <v>919</v>
+      </c>
+      <c r="H237" t="s">
+        <v>933</v>
+      </c>
+      <c r="I237" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>864</v>
       </c>
       <c r="B238" s="1">
         <v>1576</v>
       </c>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C238" t="s">
+        <v>909</v>
+      </c>
+      <c r="D238">
+        <v>31</v>
+      </c>
+      <c r="E238" t="s">
+        <v>914</v>
+      </c>
+      <c r="F238" t="s">
+        <v>919</v>
+      </c>
+      <c r="G238" t="s">
+        <v>919</v>
+      </c>
+      <c r="H238" t="s">
+        <v>933</v>
+      </c>
+      <c r="I238" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>865</v>
       </c>
       <c r="B239" s="1">
         <v>1261</v>
       </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C239" t="s">
+        <v>909</v>
+      </c>
+      <c r="D239">
+        <v>24</v>
+      </c>
+      <c r="E239" t="s">
+        <v>914</v>
+      </c>
+      <c r="F239" t="s">
+        <v>919</v>
+      </c>
+      <c r="G239" t="s">
+        <v>919</v>
+      </c>
+      <c r="H239" t="s">
+        <v>933</v>
+      </c>
+      <c r="I239" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>866</v>
       </c>
       <c r="B240" s="1">
         <v>11996</v>
       </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C240" t="s">
+        <v>909</v>
+      </c>
+      <c r="D240">
+        <v>55</v>
+      </c>
+      <c r="E240" t="s">
+        <v>914</v>
+      </c>
+      <c r="F240" t="s">
+        <v>919</v>
+      </c>
+      <c r="G240" t="s">
+        <v>919</v>
+      </c>
+      <c r="H240" t="s">
+        <v>933</v>
+      </c>
+      <c r="I240" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>867</v>
       </c>
       <c r="B241" s="1">
         <v>2296</v>
       </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C241" t="s">
+        <v>909</v>
+      </c>
+      <c r="D241">
+        <v>26</v>
+      </c>
+      <c r="E241" t="s">
+        <v>914</v>
+      </c>
+      <c r="F241" t="s">
+        <v>919</v>
+      </c>
+      <c r="G241" t="s">
+        <v>919</v>
+      </c>
+      <c r="H241" t="s">
+        <v>933</v>
+      </c>
+      <c r="I241" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>868</v>
       </c>
       <c r="B242">
         <v>422</v>
       </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C242" t="s">
+        <v>909</v>
+      </c>
+      <c r="D242">
+        <v>1</v>
+      </c>
+      <c r="E242" t="s">
+        <v>919</v>
+      </c>
+      <c r="F242" t="s">
+        <v>919</v>
+      </c>
+      <c r="G242" t="s">
+        <v>919</v>
+      </c>
+      <c r="I242" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>869</v>
       </c>
@@ -8117,7 +9549,7 @@
         <v>312159</v>
       </c>
     </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>870</v>
       </c>
@@ -8125,7 +9557,7 @@
         <v>34370</v>
       </c>
     </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>871</v>
       </c>
@@ -8133,7 +9565,7 @@
         <v>1990</v>
       </c>
     </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>872</v>
       </c>
@@ -8141,231 +9573,819 @@
         <v>3440</v>
       </c>
     </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>873</v>
       </c>
       <c r="B247" s="1">
         <v>357500</v>
       </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C247" t="s">
+        <v>950</v>
+      </c>
+      <c r="D247">
+        <v>60</v>
+      </c>
+      <c r="E247" t="s">
+        <v>914</v>
+      </c>
+      <c r="F247" t="s">
+        <v>919</v>
+      </c>
+      <c r="G247" t="s">
+        <v>919</v>
+      </c>
+      <c r="H247" t="s">
+        <v>952</v>
+      </c>
+      <c r="I247" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>130</v>
       </c>
       <c r="B248" s="1">
         <v>8929</v>
       </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C248" t="s">
+        <v>909</v>
+      </c>
+      <c r="D248">
+        <v>6</v>
+      </c>
+      <c r="E248" t="s">
+        <v>919</v>
+      </c>
+      <c r="F248" t="s">
+        <v>914</v>
+      </c>
+      <c r="G248" t="s">
+        <v>914</v>
+      </c>
+      <c r="H248" t="s">
+        <v>953</v>
+      </c>
+      <c r="I248" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>131</v>
       </c>
       <c r="B249" s="1">
         <v>6902</v>
       </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C249" t="s">
+        <v>909</v>
+      </c>
+      <c r="D249">
+        <v>6</v>
+      </c>
+      <c r="E249" t="s">
+        <v>919</v>
+      </c>
+      <c r="F249" t="s">
+        <v>914</v>
+      </c>
+      <c r="G249" t="s">
+        <v>914</v>
+      </c>
+      <c r="H249" t="s">
+        <v>953</v>
+      </c>
+      <c r="I249" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>132</v>
       </c>
       <c r="B250" s="1">
         <v>8395</v>
       </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C250" t="s">
+        <v>909</v>
+      </c>
+      <c r="D250">
+        <v>6</v>
+      </c>
+      <c r="E250" t="s">
+        <v>919</v>
+      </c>
+      <c r="F250" t="s">
+        <v>914</v>
+      </c>
+      <c r="G250" t="s">
+        <v>914</v>
+      </c>
+      <c r="H250" t="s">
+        <v>953</v>
+      </c>
+      <c r="I250" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>133</v>
       </c>
       <c r="B251" s="1">
         <v>4678</v>
       </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C251" t="s">
+        <v>909</v>
+      </c>
+      <c r="D251">
+        <v>4</v>
+      </c>
+      <c r="E251" t="s">
+        <v>914</v>
+      </c>
+      <c r="F251" t="s">
+        <v>919</v>
+      </c>
+      <c r="G251" t="s">
+        <v>919</v>
+      </c>
+      <c r="H251" t="s">
+        <v>953</v>
+      </c>
+      <c r="I251" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>134</v>
       </c>
       <c r="B252" s="1">
         <v>5378</v>
       </c>
-    </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C252" t="s">
+        <v>909</v>
+      </c>
+      <c r="D252">
+        <v>4</v>
+      </c>
+      <c r="E252" t="s">
+        <v>914</v>
+      </c>
+      <c r="F252" t="s">
+        <v>919</v>
+      </c>
+      <c r="G252" t="s">
+        <v>919</v>
+      </c>
+      <c r="H252" t="s">
+        <v>953</v>
+      </c>
+      <c r="I252" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>135</v>
       </c>
       <c r="B253" s="1">
         <v>6150</v>
       </c>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C253" t="s">
+        <v>909</v>
+      </c>
+      <c r="D253">
+        <v>4</v>
+      </c>
+      <c r="E253" t="s">
+        <v>914</v>
+      </c>
+      <c r="F253" t="s">
+        <v>919</v>
+      </c>
+      <c r="G253" t="s">
+        <v>919</v>
+      </c>
+      <c r="H253" t="s">
+        <v>953</v>
+      </c>
+      <c r="I253" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>136</v>
       </c>
       <c r="B254" s="1">
         <v>5967</v>
       </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C254" t="s">
+        <v>909</v>
+      </c>
+      <c r="D254">
+        <v>4</v>
+      </c>
+      <c r="E254" t="s">
+        <v>914</v>
+      </c>
+      <c r="F254" t="s">
+        <v>919</v>
+      </c>
+      <c r="G254" t="s">
+        <v>919</v>
+      </c>
+      <c r="H254" t="s">
+        <v>953</v>
+      </c>
+      <c r="I254" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>137</v>
       </c>
       <c r="B255" s="1">
         <v>5420</v>
       </c>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C255" t="s">
+        <v>909</v>
+      </c>
+      <c r="D255">
+        <v>4</v>
+      </c>
+      <c r="E255" t="s">
+        <v>914</v>
+      </c>
+      <c r="F255" t="s">
+        <v>919</v>
+      </c>
+      <c r="G255" t="s">
+        <v>919</v>
+      </c>
+      <c r="H255" t="s">
+        <v>953</v>
+      </c>
+      <c r="I255" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>138</v>
       </c>
       <c r="B256" s="1">
         <v>5443</v>
       </c>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C256" t="s">
+        <v>909</v>
+      </c>
+      <c r="D256">
+        <v>4</v>
+      </c>
+      <c r="E256" t="s">
+        <v>914</v>
+      </c>
+      <c r="F256" t="s">
+        <v>919</v>
+      </c>
+      <c r="G256" t="s">
+        <v>919</v>
+      </c>
+      <c r="H256" t="s">
+        <v>953</v>
+      </c>
+      <c r="I256" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>139</v>
       </c>
       <c r="B257" s="1">
         <v>19735</v>
       </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C257" t="s">
+        <v>909</v>
+      </c>
+      <c r="D257">
+        <v>21</v>
+      </c>
+      <c r="E257" t="s">
+        <v>914</v>
+      </c>
+      <c r="F257" t="s">
+        <v>919</v>
+      </c>
+      <c r="G257" t="s">
+        <v>919</v>
+      </c>
+      <c r="H257" t="s">
+        <v>953</v>
+      </c>
+      <c r="I257" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="258" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>140</v>
       </c>
       <c r="B258" s="1">
         <v>21806</v>
       </c>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C258" t="s">
+        <v>909</v>
+      </c>
+      <c r="D258">
+        <v>21</v>
+      </c>
+      <c r="E258" t="s">
+        <v>914</v>
+      </c>
+      <c r="F258" t="s">
+        <v>919</v>
+      </c>
+      <c r="G258" t="s">
+        <v>919</v>
+      </c>
+      <c r="H258" t="s">
+        <v>953</v>
+      </c>
+      <c r="I258" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="259" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>141</v>
       </c>
       <c r="B259" s="1">
         <v>24116</v>
       </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C259" t="s">
+        <v>909</v>
+      </c>
+      <c r="D259">
+        <v>21</v>
+      </c>
+      <c r="E259" t="s">
+        <v>914</v>
+      </c>
+      <c r="F259" t="s">
+        <v>919</v>
+      </c>
+      <c r="G259" t="s">
+        <v>919</v>
+      </c>
+      <c r="H259" t="s">
+        <v>953</v>
+      </c>
+      <c r="I259" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="260" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>142</v>
       </c>
       <c r="B260" s="1">
         <v>23458</v>
       </c>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C260" t="s">
+        <v>909</v>
+      </c>
+      <c r="D260">
+        <v>21</v>
+      </c>
+      <c r="E260" t="s">
+        <v>914</v>
+      </c>
+      <c r="F260" t="s">
+        <v>914</v>
+      </c>
+      <c r="G260" t="s">
+        <v>919</v>
+      </c>
+      <c r="H260" t="s">
+        <v>953</v>
+      </c>
+      <c r="I260" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="261" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>143</v>
       </c>
       <c r="B261" s="1">
         <v>20956</v>
       </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C261" t="s">
+        <v>909</v>
+      </c>
+      <c r="D261">
+        <v>21</v>
+      </c>
+      <c r="E261" t="s">
+        <v>914</v>
+      </c>
+      <c r="F261" t="s">
+        <v>919</v>
+      </c>
+      <c r="G261" t="s">
+        <v>919</v>
+      </c>
+      <c r="H261" t="s">
+        <v>953</v>
+      </c>
+      <c r="I261" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="262" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>144</v>
       </c>
       <c r="B262" s="1">
         <v>22525</v>
       </c>
-    </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C262" t="s">
+        <v>909</v>
+      </c>
+      <c r="D262">
+        <v>21</v>
+      </c>
+      <c r="E262" t="s">
+        <v>914</v>
+      </c>
+      <c r="F262" t="s">
+        <v>919</v>
+      </c>
+      <c r="G262" t="s">
+        <v>919</v>
+      </c>
+      <c r="H262" t="s">
+        <v>953</v>
+      </c>
+      <c r="I262" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="263" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>145</v>
       </c>
       <c r="B263" s="1">
         <v>11785</v>
       </c>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C263" t="s">
+        <v>909</v>
+      </c>
+      <c r="D263">
+        <v>8</v>
+      </c>
+      <c r="E263" t="s">
+        <v>914</v>
+      </c>
+      <c r="F263" t="s">
+        <v>919</v>
+      </c>
+      <c r="G263" t="s">
+        <v>919</v>
+      </c>
+      <c r="H263" t="s">
+        <v>953</v>
+      </c>
+      <c r="I263" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="264" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>146</v>
       </c>
       <c r="B264" s="1">
         <v>13416</v>
       </c>
-    </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C264" t="s">
+        <v>909</v>
+      </c>
+      <c r="D264">
+        <v>8</v>
+      </c>
+      <c r="E264" t="s">
+        <v>914</v>
+      </c>
+      <c r="F264" t="s">
+        <v>919</v>
+      </c>
+      <c r="G264" t="s">
+        <v>919</v>
+      </c>
+      <c r="H264" t="s">
+        <v>953</v>
+      </c>
+      <c r="I264" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="265" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>147</v>
       </c>
       <c r="B265" s="1">
         <v>13969</v>
       </c>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C265" t="s">
+        <v>909</v>
+      </c>
+      <c r="D265">
+        <v>8</v>
+      </c>
+      <c r="E265" t="s">
+        <v>914</v>
+      </c>
+      <c r="F265" t="s">
+        <v>919</v>
+      </c>
+      <c r="G265" t="s">
+        <v>919</v>
+      </c>
+      <c r="H265" t="s">
+        <v>953</v>
+      </c>
+      <c r="I265" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="266" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>148</v>
       </c>
       <c r="B266" s="1">
         <v>13428</v>
       </c>
-    </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C266" t="s">
+        <v>909</v>
+      </c>
+      <c r="D266">
+        <v>8</v>
+      </c>
+      <c r="E266" t="s">
+        <v>914</v>
+      </c>
+      <c r="F266" t="s">
+        <v>914</v>
+      </c>
+      <c r="G266" t="s">
+        <v>919</v>
+      </c>
+      <c r="H266" t="s">
+        <v>953</v>
+      </c>
+      <c r="I266" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>149</v>
       </c>
       <c r="B267" s="1">
         <v>13929</v>
       </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C267" t="s">
+        <v>909</v>
+      </c>
+      <c r="D267">
+        <v>8</v>
+      </c>
+      <c r="E267" t="s">
+        <v>914</v>
+      </c>
+      <c r="F267" t="s">
+        <v>919</v>
+      </c>
+      <c r="G267" t="s">
+        <v>919</v>
+      </c>
+      <c r="H267" t="s">
+        <v>953</v>
+      </c>
+      <c r="I267" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="268" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>150</v>
       </c>
       <c r="B268" s="1">
         <v>13644</v>
       </c>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C268" t="s">
+        <v>909</v>
+      </c>
+      <c r="D268">
+        <v>8</v>
+      </c>
+      <c r="E268" t="s">
+        <v>914</v>
+      </c>
+      <c r="F268" t="s">
+        <v>919</v>
+      </c>
+      <c r="G268" t="s">
+        <v>919</v>
+      </c>
+      <c r="H268" t="s">
+        <v>953</v>
+      </c>
+      <c r="I268" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="269" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>151</v>
       </c>
       <c r="B269" s="1">
         <v>23053</v>
       </c>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C269" t="s">
+        <v>909</v>
+      </c>
+      <c r="D269">
+        <v>16</v>
+      </c>
+      <c r="E269" t="s">
+        <v>914</v>
+      </c>
+      <c r="F269" t="s">
+        <v>919</v>
+      </c>
+      <c r="G269" t="s">
+        <v>919</v>
+      </c>
+      <c r="H269" t="s">
+        <v>953</v>
+      </c>
+      <c r="I269" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="270" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>152</v>
       </c>
       <c r="B270" s="1">
         <v>25837</v>
       </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C270" t="s">
+        <v>909</v>
+      </c>
+      <c r="D270">
+        <v>16</v>
+      </c>
+      <c r="E270" t="s">
+        <v>914</v>
+      </c>
+      <c r="F270" t="s">
+        <v>919</v>
+      </c>
+      <c r="G270" t="s">
+        <v>919</v>
+      </c>
+      <c r="H270" t="s">
+        <v>953</v>
+      </c>
+      <c r="I270" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="271" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>153</v>
       </c>
       <c r="B271" s="1">
         <v>27049</v>
       </c>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C271" t="s">
+        <v>909</v>
+      </c>
+      <c r="D271">
+        <v>16</v>
+      </c>
+      <c r="E271" t="s">
+        <v>914</v>
+      </c>
+      <c r="F271" t="s">
+        <v>919</v>
+      </c>
+      <c r="G271" t="s">
+        <v>919</v>
+      </c>
+      <c r="H271" t="s">
+        <v>953</v>
+      </c>
+      <c r="I271" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="272" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>154</v>
       </c>
       <c r="B272" s="1">
         <v>26011</v>
       </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C272" t="s">
+        <v>909</v>
+      </c>
+      <c r="D272">
+        <v>16</v>
+      </c>
+      <c r="E272" t="s">
+        <v>914</v>
+      </c>
+      <c r="F272" t="s">
+        <v>914</v>
+      </c>
+      <c r="G272" t="s">
+        <v>919</v>
+      </c>
+      <c r="H272" t="s">
+        <v>953</v>
+      </c>
+      <c r="I272" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>155</v>
       </c>
       <c r="B273" s="1">
         <v>26963</v>
       </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C273" t="s">
+        <v>909</v>
+      </c>
+      <c r="D273">
+        <v>16</v>
+      </c>
+      <c r="E273" t="s">
+        <v>914</v>
+      </c>
+      <c r="F273" t="s">
+        <v>919</v>
+      </c>
+      <c r="G273" t="s">
+        <v>919</v>
+      </c>
+      <c r="H273" t="s">
+        <v>953</v>
+      </c>
+      <c r="I273" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>156</v>
       </c>
       <c r="B274" s="1">
         <v>26692</v>
       </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C274" t="s">
+        <v>909</v>
+      </c>
+      <c r="D274">
+        <v>16</v>
+      </c>
+      <c r="E274" t="s">
+        <v>914</v>
+      </c>
+      <c r="F274" t="s">
+        <v>919</v>
+      </c>
+      <c r="G274" t="s">
+        <v>919</v>
+      </c>
+      <c r="H274" t="s">
+        <v>953</v>
+      </c>
+      <c r="I274" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>157</v>
       </c>
@@ -8373,7 +10393,7 @@
         <v>7602</v>
       </c>
     </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>158</v>
       </c>
@@ -8381,7 +10401,7 @@
         <v>7733</v>
       </c>
     </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>159</v>
       </c>
@@ -8389,7 +10409,7 @@
         <v>6960</v>
       </c>
     </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>160</v>
       </c>
@@ -8397,7 +10417,7 @@
         <v>3255</v>
       </c>
     </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>161</v>
       </c>
@@ -8405,7 +10425,7 @@
         <v>4509</v>
       </c>
     </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>162</v>
       </c>
@@ -8413,7 +10433,7 @@
         <v>5545</v>
       </c>
     </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>163</v>
       </c>
@@ -8421,7 +10441,7 @@
         <v>5098</v>
       </c>
     </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>164</v>
       </c>
@@ -8429,7 +10449,7 @@
         <v>5546</v>
       </c>
     </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>165</v>
       </c>
@@ -8437,7 +10457,7 @@
         <v>4286</v>
       </c>
     </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>166</v>
       </c>
@@ -8445,7 +10465,7 @@
         <v>21256</v>
       </c>
     </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>167</v>
       </c>
@@ -8453,7 +10473,7 @@
         <v>26579</v>
       </c>
     </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>168</v>
       </c>
@@ -8461,7 +10481,7 @@
         <v>29383</v>
       </c>
     </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>169</v>
       </c>
@@ -8469,7 +10489,7 @@
         <v>24919</v>
       </c>
     </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>170</v>
       </c>

</xml_diff>